<commit_message>
Refine wly backlog: merge and simplify stories
</commit_message>
<xml_diff>
--- a/product backlog template_wly.xlsx
+++ b/product backlog template_wly.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="26460" windowHeight="13300"/>
+    <workbookView windowWidth="26760" windowHeight="11480"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Story ID</t>
   </si>
@@ -62,193 +62,49 @@
     <t>DOC-J01</t>
   </si>
   <si>
-    <t>Core Class Javadoc Writing</t>
-  </si>
-  <si>
-    <t>As a backend developer,
-I want to write Oracle-standard Javadoc for all classes in model (TA/Job), service (TAService/MOJobService), and exception packages (including @author/@version/@param/@return/@throws),
-So that other team members can quickly understand code logic and reduce collaboration costs.</t>
-  </si>
-  <si>
-    <t>1. All public classes/methods have complete Javadoc with no missing key tags;
-2. Javadoc has no syntax errors and can generate HTML docs via the javadoc command;
-3. The @throws tag accurately covers all exceptions thrown by methods.</t>
-  </si>
-  <si>
-    <t>DOC-J02</t>
-  </si>
-  <si>
-    <t>Javadoc HTML Generation &amp; Optimization</t>
-  </si>
-  <si>
-    <t>As a documentation developer,
-I want to generate HTML-format Javadoc (with module indexes and search functions) and commit it to the doc folder in GitHub,
-So that reviewers can access and check documentation online without local compilation.</t>
-  </si>
-  <si>
-    <t>1. HTML docs are accessible via the root index.html file;
-2. Docs display the hierarchical relationship of core classes (e.g., model → service dependencies);
-3. GitHub preview shows no formatting errors.</t>
-  </si>
-  <si>
-    <t>DOC-J03</t>
-  </si>
-  <si>
-    <t>Javadoc Maintenance &amp; Update</t>
-  </si>
-  <si>
-    <t>As a module developer,
-I want to synchronously update Javadoc when adding new classes (e.g., AI skill-matching utility classes) in subsequent iterations,
-So that documentation remains consistent with the latest code logic and avoids misleading users.</t>
-  </si>
-  <si>
-    <t>1. Javadoc for new classes complies with the same standard as existing ones;
-2. @see tags in old docs are updated to link to new related classes;
-3. No outdated descriptions (e.g., deprecated methods marked).</t>
+    <t>Javadoc Writing &amp; Maintenance</t>
+  </si>
+  <si>
+    <t>As a backend developer, I want to write, generate, and maintain standard Javadoc for all model, service, and exception classes, so that other team members can quickly understand code logic and documentation remains consistent with updates.</t>
+  </si>
+  <si>
+    <t>1. All public classes/methods have complete Javadoc with no missing key tags. 2. Javadoc generates HTML successfully with module indexes and search. 3. Updates to new classes also update @see links. 4. No outdated or deprecated descriptions.</t>
   </si>
   <si>
     <t>DOC-U01</t>
   </si>
   <si>
-    <t>User Manual Framework Design</t>
-  </si>
-  <si>
-    <t>As a technical writer,
-I want to design a User Manual framework including "System Introduction - Role Operation Flow - FAQs - Error Prompt Explanations",
-So that end users (TA/MO/Admin) can quickly locate the guidance they need based on their roles. 1</t>
-  </si>
-  <si>
-    <t>1. Framework covers all three user roles with no missing scenarios;
-2. Chapter order aligns with user operation habits (e.g., "Registration → Job Application" for TA);
-3. Reserved placeholders for screenshots and step descriptions.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> DOC-U02</t>
-  </si>
-  <si>
-    <t>Operation Flow &amp; Screenshot Supplement</t>
-  </si>
-  <si>
-    <t>As a technical writer,
-I want to add step-by-step instructions (≤5 steps per operation) and interface screenshots (console/Web) for core actions (TA registration/MO job posting),
-So that end users can follow the manual to complete operations without additional guidance.</t>
-  </si>
-  <si>
-    <t>1. Each step description is concise (≤20 words) and uses user-friendly language;
-2. Screenshots clearly mark key elements (e.g., input boxes, "Submit" buttons);
-3. Error operations (e.g., invalid TA ID) include prompt explanations.</t>
-  </si>
-  <si>
-    <t>DOC-U03</t>
-  </si>
-  <si>
-    <t>Manual Format Unification &amp; Export</t>
-  </si>
-  <si>
-    <t>As a technical writer,
-I want to unify the User Manual into PDF format (with navigable TOC and page numbers) and control the file size ≤10MB,
-So that the manual meets project submission standards and is easy to share.</t>
-  </si>
-  <si>
-    <t>1. PDF has no formatting chaos (e.g., broken lines, misplaced images);
-2. TOC links jump to the correct pages;
-3. File is committed to the docs folder in GitHub.</t>
+    <t>User Manual Design &amp; Export</t>
+  </si>
+  <si>
+    <t>AAs a technical writer, I want to design the User Manual framework, add step-by-step operation instructions with screenshots, and export it as a PDF, so that end users (TA/MO/Admin) can easily follow and reference documentation.</t>
+  </si>
+  <si>
+    <t>1. Framework covers all three roles with no missing scenarios. 2. Each operation step is concise and clear (≤5 steps, ≤20 words). 3. Screenshots clearly mark key UI elements. 4. PDF has TOC, page numbers, and file size ≤10MB.</t>
   </si>
   <si>
     <t xml:space="preserve"> SYS-D01</t>
   </si>
   <si>
-    <t>Dialog Framework Design</t>
-  </si>
-  <si>
-    <t>As a frontend developer,
-I want to design a unified dialog interface with "menu display - user input validation - operation feedback" functions,
-So that all role menus (TA/MO/Admin) have a consistent style and reduce user learning costs.</t>
-  </si>
-  <si>
-    <t>1. Framework supports integer/string input validation (e.g., filtering non-integer menu selections);
-2. Feedback messages follow the format "[Status] Content" (e.g., "[Success] Profile created");
-3. Menus are reusable across roles.</t>
-  </si>
-  <si>
-    <t>SYS-D02</t>
-  </si>
-  <si>
-    <t>Dialog Utility Class Implementation</t>
-  </si>
-  <si>
-    <t>As a frontend developer,
-I want to develop the DialogUtil class with static methods (e.g., showMenu(), getValidIntInput(), showSuccessMessage()),
-So that interface classes can call these methods directly and avoid code redundancy.</t>
-  </si>
-  <si>
-    <t>1. All methods in DialogUtil are static and stateless;
-2. getValidIntInput() supports custom value ranges (e.g., 1-5 for menu choices);
-3. Interface classes have no duplicate dialog code.</t>
-  </si>
-  <si>
-    <t>SYS-D03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Web Dialog Adaptation </t>
-  </si>
-  <si>
-    <t>As a full-stack developer,
-I want to extend the unified dialog system to "frontend pop-up components + backend JSON responses" for Web apps,
-So that frontend-backend interaction has a consistent format and simplifies error handling.</t>
-  </si>
-  <si>
-    <t>1. Frontend pop-ups have a unified style (error/success/confirmation) with consistent colors/fonts;
-2. Backend responses use the JSON format: {"code":200,"message":"Success","data":{}};
-3. Pop-ups support dynamic content rendering.</t>
+    <t>Unified Dialog Framework &amp; Web Adaptation</t>
+  </si>
+  <si>
+    <t>As a frontend developer, I want to design a unified dialog system with reusable utility classes and adapt it for web pop-up components + backend JSON responses, so that all role menus (TA/MO/Admin) have consistent style and interaction format.</t>
+  </si>
+  <si>
+    <t>1. Framework supports input validation and feedback messages (e.g., [Success] Profile created). 2. Dialog utility class is static, reusable, and stateless. 3. Frontend pop-ups and backend JSON responses follow unified format. 4. Menus and pop-ups are reusable across roles.</t>
   </si>
   <si>
     <t xml:space="preserve"> SYS-E01</t>
   </si>
   <si>
-    <t>Exception Handler Framework Design</t>
-  </si>
-  <si>
-    <t>As a backend developer,
-I want to develop the ExceptionHandler class with unified catching/handling methods (supporting business/system/unknown exceptions),
-So that scattered try-catch blocks are eliminated and exception handling is standardized.</t>
-  </si>
-  <si>
-    <t>1. Core method handleException(Throwable e) correctly classifies exception types;
-2. Exceptions are logged to ./log/error.log with timestamps/locations;
-3. User-friendly prompts are returned (no technical jargon like "NullPointerException").</t>
-  </si>
-  <si>
-    <t>SYS-E02</t>
-  </si>
-  <si>
-    <t>Exception Integration Across Modules</t>
-  </si>
-  <si>
-    <t>As a backend developer,
-I want to call the ExceptionHandler in service/file/view layers to replace scattered try-catch code,
-So that the entire project uses the same exception handling logic and ensures consistent user prompts.</t>
-  </si>
-  <si>
-    <t>1. No scattered try-catch blocks exist in service/file/view modules;
-2. All exceptions (e.g., file read errors, invalid TA IDs) trigger consistent prompt styles;
-3. Exception logs include complete stack traces for debugging.</t>
-  </si>
-  <si>
-    <t>SYS-E03</t>
-  </si>
-  <si>
-    <t>Exception Extension &amp; Optimization</t>
-  </si>
-  <si>
-    <t>As a backend developer,
-I want to update the ExceptionHandler to support exception grading (info/warn/error) when adding new exception types (e.g., AI utility errors),
-So that different levels of exceptions are logged and prompted appropriately (e.g., "warn" for non-critical errors).</t>
-  </si>
-  <si>
-    <t>1. New exceptions (e.g., AISkillMatchException) are correctly caught and classified;
-2. Logs are stored in grade-specific files (info.log/warn.log/error.log);
-3. Prompt severity matches exception grade (e.g., red for "error").</t>
+    <t>Exception Handler Framework &amp; Optimization</t>
+  </si>
+  <si>
+    <t>As a backend developer, I want to develop and maintain a unified ExceptionHandler framework that integrates across modules and supports exception grading, so that exceptions are handled consistently and appropriately for system and business logic.</t>
+  </si>
+  <si>
+    <t>1. handleException(Throwable e) classifies exceptions correctly. 2. Logs are stored in grade-specific files (info.log/warn.log/error.log). 3. User-facing prompts are consistent and friendly. 4. New exceptions (e.g., AISkillMatchException) are integrated without breaking existing flows.</t>
   </si>
 </sst>
 </file>
@@ -261,14 +117,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -739,150 +588,150 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -892,9 +741,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="27" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1250,7 +1096,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr defaultColWidth="8.83653846153846" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="13.5096153846154" style="1" customWidth="1"/>
@@ -1297,7 +1143,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" ht="120" customHeight="1" spans="1:10">
+    <row r="2" ht="120" customHeight="1" spans="1:6">
       <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
@@ -1314,11 +1160,11 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" ht="120" customHeight="1" spans="1:10">
-      <c r="A3" s="4" t="s">
+    <row r="3" ht="120" customHeight="1" spans="1:6">
+      <c r="A3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -1331,7 +1177,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" ht="120" customHeight="1" spans="1:10">
+    <row r="4" ht="120" customHeight="1" spans="1:6">
       <c r="A4" s="5" t="s">
         <v>18</v>
       </c>
@@ -1342,17 +1188,17 @@
         <v>20</v>
       </c>
       <c r="D4" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" ht="120" customHeight="1" spans="1:10">
-      <c r="A5" s="6" t="s">
+    <row r="5" ht="120" customHeight="1" spans="1:6">
+      <c r="A5" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -1365,154 +1211,18 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" ht="120" customHeight="1" spans="1:10">
-      <c r="A6" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="1">
-        <v>1</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" ht="120" customHeight="1" spans="1:10">
-      <c r="A7" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" s="1">
-        <v>2</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" ht="120" customHeight="1" spans="1:10">
-      <c r="A8" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="1">
-        <v>1</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" ht="120" customHeight="1" spans="1:10">
-      <c r="A9" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D9" s="1">
-        <v>1</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="10" ht="120" customHeight="1" spans="1:10">
-      <c r="A10" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" s="1">
-        <v>3</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" ht="120" customHeight="1" spans="1:10">
-      <c r="A11" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D11" s="1">
-        <v>1</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="12" ht="120" customHeight="1" spans="1:10">
-      <c r="A12" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D12" s="1">
-        <v>1</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" ht="120" customHeight="1" spans="1:10">
-      <c r="A13" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D13" s="1">
-        <v>2</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
+    <row r="6" ht="120" customHeight="1"/>
+    <row r="7" ht="120" customHeight="1"/>
+    <row r="8" ht="120" customHeight="1"/>
+    <row r="9" ht="120" customHeight="1"/>
+    <row r="10" ht="120" customHeight="1"/>
+    <row r="11" ht="120" customHeight="1"/>
+    <row r="12" ht="120" customHeight="1"/>
+    <row r="13" ht="120" customHeight="1"/>
     <row r="14" ht="120" customHeight="1"/>
     <row r="15" ht="120" customHeight="1"/>
     <row r="16" ht="120" customHeight="1"/>
     <row r="17" ht="120" customHeight="1"/>
-    <row r="18" ht="120" customHeight="1"/>
-    <row r="19" ht="120" customHeight="1"/>
-    <row r="20" ht="120" customHeight="1"/>
-    <row r="21" ht="120" customHeight="1"/>
-    <row r="22" ht="120" customHeight="1"/>
-    <row r="23" ht="120" customHeight="1"/>
-    <row r="24" ht="120" customHeight="1"/>
-    <row r="25" ht="120" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>

</xml_diff>